<commit_message>
Update SBL 2026 fixtures: add Polka Dots to Women's Group B
Sixth team in W-B (Himanshi Singh & Chrisma Serrao, Sysfore). Full round-
robin in W-B grows from 10 → 15 matches; total tournament now 45 teams,
90 players, 104 matches (87 group + 17 KO). Schedule extends to 14:00.

Re-seeded SBL 2026 against the updated file. KO bracket structure unchanged
— still top-2-from-each-group → SF → Final.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/SBL_2026_Fixtures.xlsx
+++ b/data/SBL_2026_Fixtures.xlsx
@@ -763,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="26" customWidth="1" style="19" min="1" max="1"/>
@@ -824,7 +824,7 @@
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>44  (Men's Beginner: 22 | Men's Intermediate: 12 | Women's: 10)</t>
+          <t>45  (Men's Beginner: 22 | Men's Intermediate: 12 | Women's: 11)</t>
         </is>
       </c>
       <c r="C6" s="29" t="n"/>
@@ -840,7 +840,7 @@
       </c>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C7" s="29" t="n"/>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B19" s="28" t="inlineStr">
         <is>
-          <t>2 groups of 5 → Top 2 from each group = 4 teams → SF → Final</t>
+          <t>2 groups (5 + 6 teams) → Top 2 from each group = 4 teams → SF → Final</t>
         </is>
       </c>
       <c r="C19" s="29" t="n"/>
@@ -1025,7 +1025,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>09:00 - 13:40</t>
+          <t>09:00 - 14:00</t>
         </is>
       </c>
       <c r="B22" s="28" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>13:40 - 14:10</t>
+          <t>14:00 - 14:30</t>
         </is>
       </c>
       <c r="B23" s="28" t="inlineStr">
@@ -1057,7 +1057,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>14:10 - 14:45</t>
+          <t>14:30 - 15:05</t>
         </is>
       </c>
       <c r="B24" s="28" t="inlineStr">
@@ -1073,7 +1073,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>14:50 - 15:25</t>
+          <t>15:10 - 15:45</t>
         </is>
       </c>
       <c r="B25" s="28" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>15:30 - 16:05</t>
+          <t>15:50 - 16:25</t>
         </is>
       </c>
       <c r="B26" s="28" t="inlineStr">
@@ -1105,7 +1105,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>16:10 - 16:45</t>
+          <t>16:30 - 17:05</t>
         </is>
       </c>
       <c r="B27" s="28" t="inlineStr">
@@ -1121,12 +1121,12 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>16:45 - 17:00</t>
+          <t>17:05 - 17:20</t>
         </is>
       </c>
       <c r="B28" s="28" t="inlineStr">
         <is>
-          <t>Prize ceremony &amp; wrap-up</t>
+          <t>Prize ceremony &amp; wrap-up (slight overrun beyond 17:00)</t>
         </is>
       </c>
       <c r="C28" s="29" t="n"/>
@@ -1158,19 +1158,26 @@
     <row r="33">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t>• Group stage runs back-to-back on 6 courts; schedule keeps at least one slot rest between matches for any team where possible.</t>
+          <t>• Women's: Group A has 5 teams (4 matches/team); Group B has 6 teams (5 matches/team — full round-robin).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="31" t="inlineStr">
         <is>
+          <t>• Group stage runs back-to-back on 6 courts; schedule keeps at least one slot rest between matches for any team where possible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
           <t>• Knockouts use 21-point rally scoring, best of 3, cap 30. 5-minute knock-up before each KO match.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="B7:F7"/>
@@ -1185,6 +1192,7 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B17:F17"/>
@@ -1212,7 +1220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
@@ -2150,7 +2158,7 @@
     <row r="51">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>Women's — 2 groups of 5</t>
+          <t>Women's — 2 groups (5 / 6)</t>
         </is>
       </c>
     </row>
@@ -2426,6 +2434,31 @@
         </is>
       </c>
       <c r="E63" s="33" t="inlineStr">
+        <is>
+          <t>Sysfore</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="35" t="inlineStr">
+        <is>
+          <t>Group B (WB)</t>
+        </is>
+      </c>
+      <c r="B64" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" s="35" t="inlineStr">
+        <is>
+          <t>Polka Dots</t>
+        </is>
+      </c>
+      <c r="D64" s="36" t="inlineStr">
+        <is>
+          <t>Himanshi Singh &amp; Chrisma Serrao</t>
+        </is>
+      </c>
+      <c r="E64" s="35" t="inlineStr">
         <is>
           <t>Sysfore</t>
         </is>
@@ -2448,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" style="19" min="1" max="1"/>
@@ -2463,7 +2496,7 @@
     <row r="1" ht="26" customHeight="1" s="19">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>Group Stage — Master Schedule (09:00 - 13:40)</t>
+          <t>Group Stage — Master Schedule (09:00 - 14:00)</t>
         </is>
       </c>
     </row>
@@ -2770,12 +2803,12 @@
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F11" s="36" t="inlineStr">
         <is>
-          <t>Net Queens  vs  Phoenix Femmes</t>
+          <t>Racquet Rebels  vs  Power Pair</t>
         </is>
       </c>
       <c r="G11" s="35" t="inlineStr">
@@ -2840,12 +2873,12 @@
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F13" s="36" t="inlineStr">
         <is>
-          <t>Cherry Champs  vs  Prime Strikers</t>
+          <t>Polka Dots  vs  Shuttlerz</t>
         </is>
       </c>
       <c r="G13" s="35" t="inlineStr">
@@ -2905,7 +2938,7 @@
       </c>
       <c r="D15" s="35" t="inlineStr">
         <is>
-          <t>Men's Beginner</t>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E15" s="35" t="inlineStr">
@@ -2915,7 +2948,7 @@
       </c>
       <c r="F15" s="36" t="inlineStr">
         <is>
-          <t>Karnataka Knight Smashers  vs  Shuttle Pirates</t>
+          <t>Netique  vs  Double Trouble</t>
         </is>
       </c>
       <c r="G15" s="35" t="inlineStr">
@@ -2940,7 +2973,7 @@
       </c>
       <c r="D16" s="33" t="inlineStr">
         <is>
-          <t>Women's</t>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E16" s="33" t="inlineStr">
@@ -2950,7 +2983,7 @@
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
-          <t>Racquet Rebels  vs  Power Pair</t>
+          <t>Karnataka Knight Smashers  vs  Shuttle Pirates</t>
         </is>
       </c>
       <c r="G16" s="33" t="inlineStr">
@@ -2973,9 +3006,9 @@
           <t>Court 2</t>
         </is>
       </c>
-      <c r="D17" s="34" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
@@ -2985,7 +3018,7 @@
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
-          <t>Western Elite  vs  Terms &amp; Conditions</t>
+          <t>Net Queens  vs  Phoenix Femmes</t>
         </is>
       </c>
       <c r="G17" s="33" t="inlineStr">
@@ -3008,19 +3041,19 @@
           <t>Court 3</t>
         </is>
       </c>
-      <c r="D18" s="33" t="inlineStr">
-        <is>
-          <t>Women's</t>
+      <c r="D18" s="34" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F18" s="34" t="inlineStr">
         <is>
-          <t>Shuttlerz  vs  Double Trouble</t>
+          <t>Western Elite  vs  Terms &amp; Conditions</t>
         </is>
       </c>
       <c r="G18" s="33" t="inlineStr">
@@ -3043,19 +3076,19 @@
           <t>Court 4</t>
         </is>
       </c>
-      <c r="D19" s="34" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D19" s="33" t="inlineStr">
+        <is>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F19" s="34" t="inlineStr">
         <is>
-          <t>Air Strike  vs  Court Smashers</t>
+          <t>Cherry Champs  vs  Prime Strikers</t>
         </is>
       </c>
       <c r="G19" s="33" t="inlineStr">
@@ -3085,12 +3118,12 @@
       </c>
       <c r="E20" s="33" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F20" s="34" t="inlineStr">
         <is>
-          <t>Happy Hunters  vs  The Net Killers</t>
+          <t>Air Strike  vs  Court Smashers</t>
         </is>
       </c>
       <c r="G20" s="33" t="inlineStr">
@@ -3120,12 +3153,12 @@
       </c>
       <c r="E21" s="33" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F21" s="34" t="inlineStr">
         <is>
-          <t>Birdie Bandits  vs  No Mercy</t>
+          <t>Happy Hunters  vs  The Net Killers</t>
         </is>
       </c>
       <c r="G21" s="33" t="inlineStr">
@@ -3183,24 +3216,24 @@
           <t>Court 2</t>
         </is>
       </c>
-      <c r="D23" s="35" t="inlineStr">
-        <is>
-          <t>Men's Beginner</t>
+      <c r="D23" s="36" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F23" s="36" t="inlineStr">
         <is>
-          <t>Adi Poli Squad  vs  Kill Shot</t>
+          <t>Birdie Bandits  vs  No Mercy</t>
         </is>
       </c>
       <c r="G23" s="35" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
     </row>
@@ -3230,7 +3263,7 @@
       </c>
       <c r="F24" s="36" t="inlineStr">
         <is>
-          <t>Racket Machi  vs  BLUEBOX</t>
+          <t>Adi Poli Squad  vs  Kill Shot</t>
         </is>
       </c>
       <c r="G24" s="35" t="inlineStr">
@@ -3260,12 +3293,12 @@
       </c>
       <c r="E25" s="35" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F25" s="36" t="inlineStr">
         <is>
-          <t>Shuttle Strikers  vs  Dragon Boosters</t>
+          <t>Racket Machi  vs  BLUEBOX</t>
         </is>
       </c>
       <c r="G25" s="35" t="inlineStr">
@@ -3300,7 +3333,7 @@
       </c>
       <c r="F26" s="36" t="inlineStr">
         <is>
-          <t>Deadline Smashers  vs  Ice Boys</t>
+          <t>Shuttle Strikers  vs  Dragon Boosters</t>
         </is>
       </c>
       <c r="G26" s="35" t="inlineStr">
@@ -3335,7 +3368,7 @@
       </c>
       <c r="F27" s="36" t="inlineStr">
         <is>
-          <t>Net Flicks  vs  Net Ninja's</t>
+          <t>Deadline Smashers  vs  Ice Boys</t>
         </is>
       </c>
       <c r="G27" s="35" t="inlineStr">
@@ -3365,12 +3398,12 @@
       </c>
       <c r="E28" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F28" s="34" t="inlineStr">
         <is>
-          <t>Net Dominators  vs  Shuttle Smashers</t>
+          <t>Net Flicks  vs  Net Ninja's</t>
         </is>
       </c>
       <c r="G28" s="33" t="inlineStr">
@@ -3400,12 +3433,12 @@
       </c>
       <c r="E29" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
-          <t>Net Queens  vs  Cherry Champs</t>
+          <t>Racquet Rebels  vs  Polka Dots</t>
         </is>
       </c>
       <c r="G29" s="33" t="inlineStr">
@@ -3440,7 +3473,7 @@
       </c>
       <c r="F30" s="34" t="inlineStr">
         <is>
-          <t>Kamikaze  vs  The Feather Sailors</t>
+          <t>Net Dominators  vs  Shuttle Smashers</t>
         </is>
       </c>
       <c r="G30" s="33" t="inlineStr">
@@ -3470,12 +3503,12 @@
       </c>
       <c r="E31" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F31" s="34" t="inlineStr">
         <is>
-          <t>Prime Strikers  vs  Viva La Vida</t>
+          <t>Netique  vs  Power Pair</t>
         </is>
       </c>
       <c r="G31" s="33" t="inlineStr">
@@ -3505,12 +3538,12 @@
       </c>
       <c r="E32" s="33" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F32" s="34" t="inlineStr">
         <is>
-          <t>Operation SINDOOR  vs  Karnataka Knight Smashers</t>
+          <t>Kamikaze  vs  The Feather Sailors</t>
         </is>
       </c>
       <c r="G32" s="33" t="inlineStr">
@@ -3535,7 +3568,7 @@
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
-          <t>Men's Beginner</t>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E33" s="33" t="inlineStr">
@@ -3545,7 +3578,7 @@
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
-          <t>Shuttle Pirates  vs  R Squared</t>
+          <t>Double Trouble  vs  Shuttlerz</t>
         </is>
       </c>
       <c r="G33" s="33" t="inlineStr">
@@ -3570,7 +3603,7 @@
       </c>
       <c r="D34" s="35" t="inlineStr">
         <is>
-          <t>Women's</t>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E34" s="35" t="inlineStr">
@@ -3580,7 +3613,7 @@
       </c>
       <c r="F34" s="36" t="inlineStr">
         <is>
-          <t>Racquet Rebels  vs  Shuttlerz</t>
+          <t>Operation SINDOOR  vs  Karnataka Knight Smashers</t>
         </is>
       </c>
       <c r="G34" s="35" t="inlineStr">
@@ -3603,9 +3636,9 @@
           <t>Court 2</t>
         </is>
       </c>
-      <c r="D35" s="36" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D35" s="35" t="inlineStr">
+        <is>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -3615,7 +3648,7 @@
       </c>
       <c r="F35" s="36" t="inlineStr">
         <is>
-          <t>Western Elite  vs  Hire &amp; Fire</t>
+          <t>Net Queens  vs  Cherry Champs</t>
         </is>
       </c>
       <c r="G35" s="35" t="inlineStr">
@@ -3638,19 +3671,19 @@
           <t>Court 3</t>
         </is>
       </c>
-      <c r="D36" s="35" t="inlineStr">
-        <is>
-          <t>Women's</t>
+      <c r="D36" s="36" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E36" s="35" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F36" s="36" t="inlineStr">
         <is>
-          <t>Double Trouble  vs  Netique</t>
+          <t>Western Elite  vs  Hire &amp; Fire</t>
         </is>
       </c>
       <c r="G36" s="35" t="inlineStr">
@@ -3673,9 +3706,9 @@
           <t>Court 4</t>
         </is>
       </c>
-      <c r="D37" s="36" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D37" s="35" t="inlineStr">
+        <is>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
@@ -3685,7 +3718,7 @@
       </c>
       <c r="F37" s="36" t="inlineStr">
         <is>
-          <t>Air Strike  vs  Silver Li-Nings</t>
+          <t>Shuttle Pirates  vs  R Squared</t>
         </is>
       </c>
       <c r="G37" s="35" t="inlineStr">
@@ -3708,19 +3741,19 @@
           <t>Court 5</t>
         </is>
       </c>
-      <c r="D38" s="36" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D38" s="35" t="inlineStr">
+        <is>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E38" s="35" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F38" s="36" t="inlineStr">
         <is>
-          <t>Happy Hunters  vs  PaRoSmashers</t>
+          <t>Prime Strikers  vs  Viva La Vida</t>
         </is>
       </c>
       <c r="G38" s="35" t="inlineStr">
@@ -3750,12 +3783,12 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F39" s="36" t="inlineStr">
         <is>
-          <t>Birdie Bandits  vs  BREATHE</t>
+          <t>Air Strike  vs  Silver Li-Nings</t>
         </is>
       </c>
       <c r="G39" s="35" t="inlineStr">
@@ -3813,9 +3846,9 @@
           <t>Court 2</t>
         </is>
       </c>
-      <c r="D41" s="33" t="inlineStr">
-        <is>
-          <t>Men's Beginner</t>
+      <c r="D41" s="34" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E41" s="33" t="inlineStr">
@@ -3825,12 +3858,12 @@
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
-          <t>Racket Machi  vs  Ghost Riders</t>
+          <t>Happy Hunters  vs  PaRoSmashers</t>
         </is>
       </c>
       <c r="G41" s="33" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
     </row>
@@ -3860,7 +3893,7 @@
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
-          <t>BLUEBOX  vs  Kill Shot</t>
+          <t>Racket Machi  vs  Ghost Riders</t>
         </is>
       </c>
       <c r="G42" s="33" t="inlineStr">
@@ -3883,9 +3916,9 @@
           <t>Court 4</t>
         </is>
       </c>
-      <c r="D43" s="33" t="inlineStr">
-        <is>
-          <t>Men's Beginner</t>
+      <c r="D43" s="34" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E43" s="33" t="inlineStr">
@@ -3895,12 +3928,12 @@
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
-          <t>Shuttle Strikers  vs  Deadline Smashers</t>
+          <t>Birdie Bandits  vs  BREATHE</t>
         </is>
       </c>
       <c r="G43" s="33" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
     </row>
@@ -3925,12 +3958,12 @@
       </c>
       <c r="E44" s="33" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F44" s="34" t="inlineStr">
         <is>
-          <t>Net Flicks  vs  Dragon Boosters</t>
+          <t>BLUEBOX  vs  Kill Shot</t>
         </is>
       </c>
       <c r="G44" s="33" t="inlineStr">
@@ -3965,7 +3998,7 @@
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
-          <t>Net Ninja's  vs  Ice Boys</t>
+          <t>Shuttle Strikers  vs  Deadline Smashers</t>
         </is>
       </c>
       <c r="G45" s="33" t="inlineStr">
@@ -3995,12 +4028,12 @@
       </c>
       <c r="E46" s="35" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F46" s="36" t="inlineStr">
         <is>
-          <t>Net Dominators  vs  Kamikaze</t>
+          <t>Net Flicks  vs  Dragon Boosters</t>
         </is>
       </c>
       <c r="G46" s="35" t="inlineStr">
@@ -4030,12 +4063,12 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F47" s="36" t="inlineStr">
         <is>
-          <t>Net Queens  vs  Prime Strikers</t>
+          <t>Racquet Rebels  vs  Netique</t>
         </is>
       </c>
       <c r="G47" s="35" t="inlineStr">
@@ -4065,12 +4098,12 @@
       </c>
       <c r="E48" s="35" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F48" s="36" t="inlineStr">
         <is>
-          <t>Phantom Nemesis  vs  The Feather Sailors</t>
+          <t>Net Ninja's  vs  Ice Boys</t>
         </is>
       </c>
       <c r="G48" s="35" t="inlineStr">
@@ -4100,12 +4133,12 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F49" s="36" t="inlineStr">
         <is>
-          <t>Phoenix Femmes  vs  Viva La Vida</t>
+          <t>Double Trouble  vs  Polka Dots</t>
         </is>
       </c>
       <c r="G49" s="35" t="inlineStr">
@@ -4135,12 +4168,12 @@
       </c>
       <c r="E50" s="35" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F50" s="36" t="inlineStr">
         <is>
-          <t>Operation SINDOOR  vs  Shuttle Pirates</t>
+          <t>Net Dominators  vs  Kamikaze</t>
         </is>
       </c>
       <c r="G50" s="35" t="inlineStr">
@@ -4165,7 +4198,7 @@
       </c>
       <c r="D51" s="35" t="inlineStr">
         <is>
-          <t>Men's Beginner</t>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
@@ -4175,7 +4208,7 @@
       </c>
       <c r="F51" s="36" t="inlineStr">
         <is>
-          <t>Team Masala Dosa  vs  R Squared</t>
+          <t>Shuttlerz  vs  Power Pair</t>
         </is>
       </c>
       <c r="G51" s="35" t="inlineStr">
@@ -4200,7 +4233,7 @@
       </c>
       <c r="D52" s="33" t="inlineStr">
         <is>
-          <t>Women's</t>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E52" s="33" t="inlineStr">
@@ -4210,7 +4243,7 @@
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
-          <t>Racquet Rebels  vs  Double Trouble</t>
+          <t>Operation SINDOOR  vs  Shuttle Pirates</t>
         </is>
       </c>
       <c r="G52" s="33" t="inlineStr">
@@ -4233,9 +4266,9 @@
           <t>Court 2</t>
         </is>
       </c>
-      <c r="D53" s="34" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D53" s="33" t="inlineStr">
+        <is>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E53" s="33" t="inlineStr">
@@ -4245,7 +4278,7 @@
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
-          <t>Terms &amp; Conditions  vs  Hire &amp; Fire</t>
+          <t>Net Queens  vs  Prime Strikers</t>
         </is>
       </c>
       <c r="G53" s="33" t="inlineStr">
@@ -4268,19 +4301,19 @@
           <t>Court 3</t>
         </is>
       </c>
-      <c r="D54" s="33" t="inlineStr">
-        <is>
-          <t>Women's</t>
+      <c r="D54" s="34" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E54" s="33" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
-          <t>Power Pair  vs  Netique</t>
+          <t>Terms &amp; Conditions  vs  Hire &amp; Fire</t>
         </is>
       </c>
       <c r="G54" s="33" t="inlineStr">
@@ -4303,9 +4336,9 @@
           <t>Court 4</t>
         </is>
       </c>
-      <c r="D55" s="34" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D55" s="33" t="inlineStr">
+        <is>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E55" s="33" t="inlineStr">
@@ -4315,7 +4348,7 @@
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
-          <t>Court Smashers  vs  Silver Li-Nings</t>
+          <t>Team Masala Dosa  vs  R Squared</t>
         </is>
       </c>
       <c r="G55" s="33" t="inlineStr">
@@ -4338,19 +4371,19 @@
           <t>Court 5</t>
         </is>
       </c>
-      <c r="D56" s="34" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D56" s="33" t="inlineStr">
+        <is>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E56" s="33" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
-          <t>The Net Killers  vs  PaRoSmashers</t>
+          <t>Phoenix Femmes  vs  Viva La Vida</t>
         </is>
       </c>
       <c r="G56" s="33" t="inlineStr">
@@ -4373,19 +4406,19 @@
           <t>Court 6</t>
         </is>
       </c>
-      <c r="D57" s="34" t="inlineStr">
-        <is>
-          <t>Men's Intermediate</t>
+      <c r="D57" s="33" t="inlineStr">
+        <is>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E57" s="33" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
-          <t>No Mercy  vs  BREATHE</t>
+          <t>Phantom Nemesis  vs  The Feather Sailors</t>
         </is>
       </c>
       <c r="G57" s="33" t="inlineStr">
@@ -4443,24 +4476,24 @@
           <t>Court 2</t>
         </is>
       </c>
-      <c r="D59" s="35" t="inlineStr">
-        <is>
-          <t>Men's Beginner</t>
+      <c r="D59" s="36" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F59" s="36" t="inlineStr">
         <is>
-          <t>BLUEBOX  vs  Adi Poli Squad</t>
+          <t>Court Smashers  vs  Silver Li-Nings</t>
         </is>
       </c>
       <c r="G59" s="35" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
@@ -4490,7 +4523,7 @@
       </c>
       <c r="F60" s="36" t="inlineStr">
         <is>
-          <t>Ghost Riders  vs  Kill Shot</t>
+          <t>BLUEBOX  vs  Adi Poli Squad</t>
         </is>
       </c>
       <c r="G60" s="35" t="inlineStr">
@@ -4513,24 +4546,24 @@
           <t>Court 4</t>
         </is>
       </c>
-      <c r="D61" s="35" t="inlineStr">
-        <is>
-          <t>Men's Beginner</t>
+      <c r="D61" s="36" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F61" s="36" t="inlineStr">
         <is>
-          <t>Shuttle Strikers  vs  Net Flicks</t>
+          <t>The Net Killers  vs  PaRoSmashers</t>
         </is>
       </c>
       <c r="G61" s="35" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
@@ -4555,12 +4588,12 @@
       </c>
       <c r="E62" s="35" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F62" s="36" t="inlineStr">
         <is>
-          <t>Net Ninja's  vs  Deadline Smashers</t>
+          <t>Ghost Riders  vs  Kill Shot</t>
         </is>
       </c>
       <c r="G62" s="35" t="inlineStr">
@@ -4583,9 +4616,9 @@
           <t>Court 6</t>
         </is>
       </c>
-      <c r="D63" s="35" t="inlineStr">
-        <is>
-          <t>Men's Beginner</t>
+      <c r="D63" s="36" t="inlineStr">
+        <is>
+          <t>Men's Intermediate</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
@@ -4595,12 +4628,12 @@
       </c>
       <c r="F63" s="36" t="inlineStr">
         <is>
-          <t>Dragon Boosters  vs  Ice Boys</t>
+          <t>No Mercy  vs  BREATHE</t>
         </is>
       </c>
       <c r="G63" s="35" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
@@ -4625,12 +4658,12 @@
       </c>
       <c r="E64" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
-          <t>Net Dominators  vs  The Feather Sailors</t>
+          <t>Shuttle Strikers  vs  Net Flicks</t>
         </is>
       </c>
       <c r="G64" s="33" t="inlineStr">
@@ -4660,12 +4693,12 @@
       </c>
       <c r="E65" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
-          <t>Net Queens  vs  Viva La Vida</t>
+          <t>Racquet Rebels  vs  Double Trouble</t>
         </is>
       </c>
       <c r="G65" s="33" t="inlineStr">
@@ -4695,12 +4728,12 @@
       </c>
       <c r="E66" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
-          <t>Phantom Nemesis  vs  Shuttle Smashers</t>
+          <t>Net Ninja's  vs  Deadline Smashers</t>
         </is>
       </c>
       <c r="G66" s="33" t="inlineStr">
@@ -4730,12 +4763,12 @@
       </c>
       <c r="E67" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
-          <t>Phoenix Femmes  vs  Cherry Champs</t>
+          <t>Shuttlerz  vs  Netique</t>
         </is>
       </c>
       <c r="G67" s="33" t="inlineStr">
@@ -4765,12 +4798,12 @@
       </c>
       <c r="E68" s="33" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
-          <t>Operation SINDOOR  vs  R Squared</t>
+          <t>Dragon Boosters  vs  Ice Boys</t>
         </is>
       </c>
       <c r="G68" s="33" t="inlineStr">
@@ -4795,7 +4828,7 @@
       </c>
       <c r="D69" s="33" t="inlineStr">
         <is>
-          <t>Men's Beginner</t>
+          <t>Women's</t>
         </is>
       </c>
       <c r="E69" s="33" t="inlineStr">
@@ -4805,7 +4838,7 @@
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
-          <t>Team Masala Dosa  vs  Karnataka Knight Smashers</t>
+          <t>Polka Dots  vs  Power Pair</t>
         </is>
       </c>
       <c r="G69" s="33" t="inlineStr">
@@ -4835,17 +4868,17 @@
       </c>
       <c r="E70" s="35" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F70" s="36" t="inlineStr">
         <is>
-          <t>Faulty Servers  vs  BLUEBOX</t>
+          <t>Net Dominators  vs  The Feather Sailors</t>
         </is>
       </c>
       <c r="G70" s="35" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
@@ -4870,12 +4903,12 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F71" s="36" t="inlineStr">
         <is>
-          <t>Racquet Rebels  vs  Netique</t>
+          <t>Net Queens  vs  Viva La Vida</t>
         </is>
       </c>
       <c r="G71" s="35" t="inlineStr">
@@ -4905,17 +4938,17 @@
       </c>
       <c r="E72" s="35" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F72" s="36" t="inlineStr">
         <is>
-          <t>Kill Shot  vs  Racket Machi</t>
+          <t>Phantom Nemesis  vs  Shuttle Smashers</t>
         </is>
       </c>
       <c r="G72" s="35" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
@@ -4940,12 +4973,12 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F73" s="36" t="inlineStr">
         <is>
-          <t>Power Pair  vs  Shuttlerz</t>
+          <t>Phoenix Femmes  vs  Cherry Champs</t>
         </is>
       </c>
       <c r="G73" s="35" t="inlineStr">
@@ -4975,17 +5008,17 @@
       </c>
       <c r="E74" s="35" t="inlineStr">
         <is>
-          <t>Group C</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F74" s="36" t="inlineStr">
         <is>
-          <t>Ghost Riders  vs  Adi Poli Squad</t>
+          <t>Operation SINDOOR  vs  R Squared</t>
         </is>
       </c>
       <c r="G74" s="35" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
@@ -5010,17 +5043,17 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Group D</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F75" s="36" t="inlineStr">
         <is>
-          <t>Shuttle Strikers  vs  Net Ninja's</t>
+          <t>Team Masala Dosa  vs  Karnataka Knight Smashers</t>
         </is>
       </c>
       <c r="G75" s="35" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
@@ -5045,12 +5078,12 @@
       </c>
       <c r="E76" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
-          <t>Phantom Nemesis  vs  Kamikaze</t>
+          <t>Faulty Servers  vs  BLUEBOX</t>
         </is>
       </c>
       <c r="G76" s="33" t="inlineStr">
@@ -5080,12 +5113,12 @@
       </c>
       <c r="E77" s="33" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
-          <t>Shuttle Smashers  vs  The Feather Sailors</t>
+          <t>Kill Shot  vs  Racket Machi</t>
         </is>
       </c>
       <c r="G77" s="33" t="inlineStr">
@@ -5115,12 +5148,12 @@
       </c>
       <c r="E78" s="33" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group C</t>
         </is>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
-          <t>Team Masala Dosa  vs  Shuttle Pirates</t>
+          <t>Ghost Riders  vs  Adi Poli Squad</t>
         </is>
       </c>
       <c r="G78" s="33" t="inlineStr">
@@ -5150,12 +5183,12 @@
       </c>
       <c r="E79" s="33" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group D</t>
         </is>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
-          <t>Karnataka Knight Smashers  vs  R Squared</t>
+          <t>Shuttle Strikers  vs  Net Ninja's</t>
         </is>
       </c>
       <c r="G79" s="33" t="inlineStr">
@@ -5250,7 +5283,7 @@
       </c>
       <c r="D82" s="35" t="inlineStr">
         <is>
-          <t>Women's</t>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E82" s="35" t="inlineStr">
@@ -5260,7 +5293,7 @@
       </c>
       <c r="F82" s="36" t="inlineStr">
         <is>
-          <t>Phoenix Femmes  vs  Prime Strikers</t>
+          <t>Phantom Nemesis  vs  Kamikaze</t>
         </is>
       </c>
       <c r="G82" s="35" t="inlineStr">
@@ -5290,12 +5323,12 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Group A</t>
+          <t>Group B</t>
         </is>
       </c>
       <c r="F83" s="36" t="inlineStr">
         <is>
-          <t>Cherry Champs  vs  Viva La Vida</t>
+          <t>Racquet Rebels  vs  Shuttlerz</t>
         </is>
       </c>
       <c r="G83" s="35" t="inlineStr">
@@ -5320,17 +5353,17 @@
       </c>
       <c r="D84" s="35" t="inlineStr">
         <is>
-          <t>Women's</t>
+          <t>Men's Beginner</t>
         </is>
       </c>
       <c r="E84" s="35" t="inlineStr">
         <is>
-          <t>Group B</t>
+          <t>Group A</t>
         </is>
       </c>
       <c r="F84" s="36" t="inlineStr">
         <is>
-          <t>Power Pair  vs  Double Trouble</t>
+          <t>Shuttle Smashers  vs  The Feather Sailors</t>
         </is>
       </c>
       <c r="G84" s="35" t="inlineStr">
@@ -5365,10 +5398,185 @@
       </c>
       <c r="F85" s="36" t="inlineStr">
         <is>
-          <t>Shuttlerz  vs  Netique</t>
+          <t>Power Pair  vs  Double Trouble</t>
         </is>
       </c>
       <c r="G85" s="35" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="35" t="n">
+        <v>14</v>
+      </c>
+      <c r="B86" s="35" t="inlineStr">
+        <is>
+          <t>13:20 - 13:40</t>
+        </is>
+      </c>
+      <c r="C86" s="35" t="inlineStr">
+        <is>
+          <t>Court 5</t>
+        </is>
+      </c>
+      <c r="D86" s="35" t="inlineStr">
+        <is>
+          <t>Men's Beginner</t>
+        </is>
+      </c>
+      <c r="E86" s="35" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="F86" s="36" t="inlineStr">
+        <is>
+          <t>Team Masala Dosa  vs  Shuttle Pirates</t>
+        </is>
+      </c>
+      <c r="G86" s="35" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="35" t="n">
+        <v>14</v>
+      </c>
+      <c r="B87" s="35" t="inlineStr">
+        <is>
+          <t>13:20 - 13:40</t>
+        </is>
+      </c>
+      <c r="C87" s="35" t="inlineStr">
+        <is>
+          <t>Court 6</t>
+        </is>
+      </c>
+      <c r="D87" s="35" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="E87" s="35" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="F87" s="36" t="inlineStr">
+        <is>
+          <t>Polka Dots  vs  Netique</t>
+        </is>
+      </c>
+      <c r="G87" s="35" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="B88" s="33" t="inlineStr">
+        <is>
+          <t>13:40 - 14:00</t>
+        </is>
+      </c>
+      <c r="C88" s="33" t="inlineStr">
+        <is>
+          <t>Court 1</t>
+        </is>
+      </c>
+      <c r="D88" s="33" t="inlineStr">
+        <is>
+          <t>Men's Beginner</t>
+        </is>
+      </c>
+      <c r="E88" s="33" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="F88" s="34" t="inlineStr">
+        <is>
+          <t>Karnataka Knight Smashers  vs  R Squared</t>
+        </is>
+      </c>
+      <c r="G88" s="33" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="B89" s="33" t="inlineStr">
+        <is>
+          <t>13:40 - 14:00</t>
+        </is>
+      </c>
+      <c r="C89" s="33" t="inlineStr">
+        <is>
+          <t>Court 2</t>
+        </is>
+      </c>
+      <c r="D89" s="33" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="E89" s="33" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="F89" s="34" t="inlineStr">
+        <is>
+          <t>Phoenix Femmes  vs  Prime Strikers</t>
+        </is>
+      </c>
+      <c r="G89" s="33" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="B90" s="33" t="inlineStr">
+        <is>
+          <t>13:40 - 14:00</t>
+        </is>
+      </c>
+      <c r="C90" s="33" t="inlineStr">
+        <is>
+          <t>Court 3</t>
+        </is>
+      </c>
+      <c r="D90" s="33" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="E90" s="33" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="F90" s="34" t="inlineStr">
+        <is>
+          <t>Cherry Champs  vs  Viva La Vida</t>
+        </is>
+      </c>
+      <c r="G90" s="33" t="inlineStr">
         <is>
           <t>R5</t>
         </is>
@@ -5388,7 +5596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" style="19" min="1" max="1"/>
@@ -5411,7 +5619,7 @@
     <row r="3">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>Group Stage (09:00 - 13:40)</t>
+          <t>Group Stage (09:00 - 14:00)</t>
         </is>
       </c>
     </row>
@@ -5513,7 +5721,7 @@
       </c>
       <c r="D6" s="36" t="inlineStr">
         <is>
-          <t>[W-A R1] Net Queens vs Phoenix Femmes</t>
+          <t>[W-B R1] Racquet Rebels vs Power Pair</t>
         </is>
       </c>
       <c r="E6" s="36" t="inlineStr">
@@ -5523,7 +5731,7 @@
       </c>
       <c r="F6" s="36" t="inlineStr">
         <is>
-          <t>[W-A R1] Cherry Champs vs Prime Strikers</t>
+          <t>[W-B R1] Polka Dots vs Shuttlerz</t>
         </is>
       </c>
       <c r="G6" s="36" t="inlineStr">
@@ -5533,7 +5741,7 @@
       </c>
       <c r="H6" s="36" t="inlineStr">
         <is>
-          <t>[MB-B R1] Karnataka Knight Smashers vs Shuttle Pirates</t>
+          <t>[W-B R1] Netique vs Double Trouble</t>
         </is>
       </c>
     </row>
@@ -5548,32 +5756,32 @@
       </c>
       <c r="C7" s="34" t="inlineStr">
         <is>
-          <t>[W-B R1] Racquet Rebels vs Power Pair</t>
+          <t>[MB-B R1] Karnataka Knight Smashers vs Shuttle Pirates</t>
         </is>
       </c>
       <c r="D7" s="34" t="inlineStr">
         <is>
+          <t>[W-A R1] Net Queens vs Phoenix Femmes</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
           <t>[MI-A R1] Western Elite vs Terms &amp; Conditions</t>
         </is>
       </c>
-      <c r="E7" s="34" t="inlineStr">
-        <is>
-          <t>[W-B R1] Shuttlerz vs Double Trouble</t>
-        </is>
-      </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
+          <t>[W-A R1] Cherry Champs vs Prime Strikers</t>
+        </is>
+      </c>
+      <c r="G7" s="34" t="inlineStr">
+        <is>
           <t>[MI-B R1] Air Strike vs Court Smashers</t>
         </is>
       </c>
-      <c r="G7" s="34" t="inlineStr">
+      <c r="H7" s="34" t="inlineStr">
         <is>
           <t>[MI-C R1] Happy Hunters vs The Net Killers</t>
-        </is>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>[MI-D R1] Birdie Bandits vs No Mercy</t>
         </is>
       </c>
     </row>
@@ -5593,27 +5801,27 @@
       </c>
       <c r="D8" s="36" t="inlineStr">
         <is>
+          <t>[MI-D R1] Birdie Bandits vs No Mercy</t>
+        </is>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
           <t>[MB-C R2] Adi Poli Squad vs Kill Shot</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr">
+      <c r="F8" s="36" t="inlineStr">
         <is>
           <t>[MB-C R2] Racket Machi vs BLUEBOX</t>
         </is>
       </c>
-      <c r="F8" s="36" t="inlineStr">
+      <c r="G8" s="36" t="inlineStr">
         <is>
           <t>[MB-D R2] Shuttle Strikers vs Dragon Boosters</t>
         </is>
       </c>
-      <c r="G8" s="36" t="inlineStr">
+      <c r="H8" s="36" t="inlineStr">
         <is>
           <t>[MB-D R2] Deadline Smashers vs Ice Boys</t>
-        </is>
-      </c>
-      <c r="H8" s="36" t="inlineStr">
-        <is>
-          <t>[MB-D R2] Net Flicks vs Net Ninja's</t>
         </is>
       </c>
     </row>
@@ -5628,32 +5836,32 @@
       </c>
       <c r="C9" s="34" t="inlineStr">
         <is>
+          <t>[MB-D R2] Net Flicks vs Net Ninja's</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="inlineStr">
+        <is>
+          <t>[W-B R2] Racquet Rebels vs Polka Dots</t>
+        </is>
+      </c>
+      <c r="E9" s="34" t="inlineStr">
+        <is>
           <t>[MB-A R2] Net Dominators vs Shuttle Smashers</t>
         </is>
       </c>
-      <c r="D9" s="34" t="inlineStr">
-        <is>
-          <t>[W-A R2] Net Queens vs Cherry Champs</t>
-        </is>
-      </c>
-      <c r="E9" s="34" t="inlineStr">
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>[W-B R2] Netique vs Power Pair</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
         <is>
           <t>[MB-A R2] Kamikaze vs The Feather Sailors</t>
         </is>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>[W-A R2] Prime Strikers vs Viva La Vida</t>
-        </is>
-      </c>
-      <c r="G9" s="34" t="inlineStr">
-        <is>
-          <t>[MB-B R2] Operation SINDOOR vs Karnataka Knight Smashers</t>
-        </is>
-      </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
-          <t>[MB-B R2] Shuttle Pirates vs R Squared</t>
+          <t>[W-B R2] Double Trouble vs Shuttlerz</t>
         </is>
       </c>
     </row>
@@ -5668,32 +5876,32 @@
       </c>
       <c r="C10" s="36" t="inlineStr">
         <is>
-          <t>[W-B R2] Racquet Rebels vs Shuttlerz</t>
+          <t>[MB-B R2] Operation SINDOOR vs Karnataka Knight Smashers</t>
         </is>
       </c>
       <c r="D10" s="36" t="inlineStr">
         <is>
+          <t>[W-A R2] Net Queens vs Cherry Champs</t>
+        </is>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
           <t>[MI-A R2] Western Elite vs Hire &amp; Fire</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>[W-B R2] Double Trouble vs Netique</t>
-        </is>
-      </c>
       <c r="F10" s="36" t="inlineStr">
         <is>
+          <t>[MB-B R2] Shuttle Pirates vs R Squared</t>
+        </is>
+      </c>
+      <c r="G10" s="36" t="inlineStr">
+        <is>
+          <t>[W-A R2] Prime Strikers vs Viva La Vida</t>
+        </is>
+      </c>
+      <c r="H10" s="36" t="inlineStr">
+        <is>
           <t>[MI-B R2] Air Strike vs Silver Li-Nings</t>
-        </is>
-      </c>
-      <c r="G10" s="36" t="inlineStr">
-        <is>
-          <t>[MI-C R2] Happy Hunters vs PaRoSmashers</t>
-        </is>
-      </c>
-      <c r="H10" s="36" t="inlineStr">
-        <is>
-          <t>[MI-D R2] Birdie Bandits vs BREATHE</t>
         </is>
       </c>
     </row>
@@ -5713,27 +5921,27 @@
       </c>
       <c r="D11" s="34" t="inlineStr">
         <is>
+          <t>[MI-C R2] Happy Hunters vs PaRoSmashers</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
           <t>[MB-C R3] Racket Machi vs Ghost Riders</t>
         </is>
       </c>
-      <c r="E11" s="34" t="inlineStr">
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>[MI-D R2] Birdie Bandits vs BREATHE</t>
+        </is>
+      </c>
+      <c r="G11" s="34" t="inlineStr">
         <is>
           <t>[MB-C R3] BLUEBOX vs Kill Shot</t>
         </is>
       </c>
-      <c r="F11" s="34" t="inlineStr">
+      <c r="H11" s="34" t="inlineStr">
         <is>
           <t>[MB-D R3] Shuttle Strikers vs Deadline Smashers</t>
-        </is>
-      </c>
-      <c r="G11" s="34" t="inlineStr">
-        <is>
-          <t>[MB-D R3] Net Flicks vs Dragon Boosters</t>
-        </is>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>[MB-D R3] Net Ninja's vs Ice Boys</t>
         </is>
       </c>
     </row>
@@ -5748,32 +5956,32 @@
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
+          <t>[MB-D R3] Net Flicks vs Dragon Boosters</t>
+        </is>
+      </c>
+      <c r="D12" s="36" t="inlineStr">
+        <is>
+          <t>[W-B R3] Racquet Rebels vs Netique</t>
+        </is>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>[MB-D R3] Net Ninja's vs Ice Boys</t>
+        </is>
+      </c>
+      <c r="F12" s="36" t="inlineStr">
+        <is>
+          <t>[W-B R3] Double Trouble vs Polka Dots</t>
+        </is>
+      </c>
+      <c r="G12" s="36" t="inlineStr">
+        <is>
           <t>[MB-A R3] Net Dominators vs Kamikaze</t>
         </is>
       </c>
-      <c r="D12" s="36" t="inlineStr">
-        <is>
-          <t>[W-A R3] Net Queens vs Prime Strikers</t>
-        </is>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>[MB-A R3] Phantom Nemesis vs The Feather Sailors</t>
-        </is>
-      </c>
-      <c r="F12" s="36" t="inlineStr">
-        <is>
-          <t>[W-A R3] Phoenix Femmes vs Viva La Vida</t>
-        </is>
-      </c>
-      <c r="G12" s="36" t="inlineStr">
-        <is>
-          <t>[MB-B R3] Operation SINDOOR vs Shuttle Pirates</t>
-        </is>
-      </c>
       <c r="H12" s="36" t="inlineStr">
         <is>
-          <t>[MB-B R3] Team Masala Dosa vs R Squared</t>
+          <t>[W-B R3] Shuttlerz vs Power Pair</t>
         </is>
       </c>
     </row>
@@ -5788,32 +5996,32 @@
       </c>
       <c r="C13" s="34" t="inlineStr">
         <is>
-          <t>[W-B R3] Racquet Rebels vs Double Trouble</t>
+          <t>[MB-B R3] Operation SINDOOR vs Shuttle Pirates</t>
         </is>
       </c>
       <c r="D13" s="34" t="inlineStr">
         <is>
+          <t>[W-A R3] Net Queens vs Prime Strikers</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
           <t>[MI-A R3] Terms &amp; Conditions vs Hire &amp; Fire</t>
         </is>
       </c>
-      <c r="E13" s="34" t="inlineStr">
-        <is>
-          <t>[W-B R3] Power Pair vs Netique</t>
-        </is>
-      </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
-          <t>[MI-B R3] Court Smashers vs Silver Li-Nings</t>
+          <t>[MB-B R3] Team Masala Dosa vs R Squared</t>
         </is>
       </c>
       <c r="G13" s="34" t="inlineStr">
         <is>
-          <t>[MI-C R3] The Net Killers vs PaRoSmashers</t>
+          <t>[W-A R3] Phoenix Femmes vs Viva La Vida</t>
         </is>
       </c>
       <c r="H13" s="34" t="inlineStr">
         <is>
-          <t>[MI-D R3] No Mercy vs BREATHE</t>
+          <t>[MB-A R3] Phantom Nemesis vs The Feather Sailors</t>
         </is>
       </c>
     </row>
@@ -5833,27 +6041,27 @@
       </c>
       <c r="D14" s="36" t="inlineStr">
         <is>
+          <t>[MI-B R3] Court Smashers vs Silver Li-Nings</t>
+        </is>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
           <t>[MB-C R4] BLUEBOX vs Adi Poli Squad</t>
         </is>
       </c>
-      <c r="E14" s="36" t="inlineStr">
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>[MI-C R3] The Net Killers vs PaRoSmashers</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
         <is>
           <t>[MB-C R4] Ghost Riders vs Kill Shot</t>
         </is>
       </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>[MB-D R4] Shuttle Strikers vs Net Flicks</t>
-        </is>
-      </c>
-      <c r="G14" s="36" t="inlineStr">
-        <is>
-          <t>[MB-D R4] Net Ninja's vs Deadline Smashers</t>
-        </is>
-      </c>
       <c r="H14" s="36" t="inlineStr">
         <is>
-          <t>[MB-D R4] Dragon Boosters vs Ice Boys</t>
+          <t>[MI-D R3] No Mercy vs BREATHE</t>
         </is>
       </c>
     </row>
@@ -5868,32 +6076,32 @@
       </c>
       <c r="C15" s="34" t="inlineStr">
         <is>
-          <t>[MB-A R4] Net Dominators vs The Feather Sailors</t>
+          <t>[MB-D R4] Shuttle Strikers vs Net Flicks</t>
         </is>
       </c>
       <c r="D15" s="34" t="inlineStr">
         <is>
-          <t>[W-A R4] Net Queens vs Viva La Vida</t>
+          <t>[W-B R4] Racquet Rebels vs Double Trouble</t>
         </is>
       </c>
       <c r="E15" s="34" t="inlineStr">
         <is>
-          <t>[MB-A R4] Phantom Nemesis vs Shuttle Smashers</t>
+          <t>[MB-D R4] Net Ninja's vs Deadline Smashers</t>
         </is>
       </c>
       <c r="F15" s="34" t="inlineStr">
         <is>
-          <t>[W-A R4] Phoenix Femmes vs Cherry Champs</t>
+          <t>[W-B R4] Shuttlerz vs Netique</t>
         </is>
       </c>
       <c r="G15" s="34" t="inlineStr">
         <is>
-          <t>[MB-B R4] Operation SINDOOR vs R Squared</t>
+          <t>[MB-D R4] Dragon Boosters vs Ice Boys</t>
         </is>
       </c>
       <c r="H15" s="34" t="inlineStr">
         <is>
-          <t>[MB-B R4] Team Masala Dosa vs Karnataka Knight Smashers</t>
+          <t>[W-B R4] Polka Dots vs Power Pair</t>
         </is>
       </c>
     </row>
@@ -5908,32 +6116,32 @@
       </c>
       <c r="C16" s="36" t="inlineStr">
         <is>
-          <t>[MB-C R5] Faulty Servers vs BLUEBOX</t>
+          <t>[MB-A R4] Net Dominators vs The Feather Sailors</t>
         </is>
       </c>
       <c r="D16" s="36" t="inlineStr">
         <is>
-          <t>[W-B R4] Racquet Rebels vs Netique</t>
+          <t>[W-A R4] Net Queens vs Viva La Vida</t>
         </is>
       </c>
       <c r="E16" s="36" t="inlineStr">
         <is>
-          <t>[MB-C R5] Kill Shot vs Racket Machi</t>
+          <t>[MB-A R4] Phantom Nemesis vs Shuttle Smashers</t>
         </is>
       </c>
       <c r="F16" s="36" t="inlineStr">
         <is>
-          <t>[W-B R4] Power Pair vs Shuttlerz</t>
+          <t>[W-A R4] Phoenix Femmes vs Cherry Champs</t>
         </is>
       </c>
       <c r="G16" s="36" t="inlineStr">
         <is>
-          <t>[MB-C R5] Ghost Riders vs Adi Poli Squad</t>
+          <t>[MB-B R4] Operation SINDOOR vs R Squared</t>
         </is>
       </c>
       <c r="H16" s="36" t="inlineStr">
         <is>
-          <t>[MB-D R5] Shuttle Strikers vs Net Ninja's</t>
+          <t>[MB-B R4] Team Masala Dosa vs Karnataka Knight Smashers</t>
         </is>
       </c>
     </row>
@@ -5948,22 +6156,22 @@
       </c>
       <c r="C17" s="34" t="inlineStr">
         <is>
-          <t>[MB-A R5] Phantom Nemesis vs Kamikaze</t>
+          <t>[MB-C R5] Faulty Servers vs BLUEBOX</t>
         </is>
       </c>
       <c r="D17" s="34" t="inlineStr">
         <is>
-          <t>[MB-A R5] Shuttle Smashers vs The Feather Sailors</t>
+          <t>[MB-C R5] Kill Shot vs Racket Machi</t>
         </is>
       </c>
       <c r="E17" s="34" t="inlineStr">
         <is>
-          <t>[MB-B R5] Team Masala Dosa vs Shuttle Pirates</t>
+          <t>[MB-C R5] Ghost Riders vs Adi Poli Squad</t>
         </is>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
-          <t>[MB-B R5] Karnataka Knight Smashers vs R Squared</t>
+          <t>[MB-D R5] Shuttle Strikers vs Net Ninja's</t>
         </is>
       </c>
       <c r="G17" s="34" t="inlineStr">
@@ -5988,230 +6196,266 @@
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
+          <t>[MB-A R5] Phantom Nemesis vs Kamikaze</t>
+        </is>
+      </c>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>[W-B R5] Racquet Rebels vs Shuttlerz</t>
+        </is>
+      </c>
+      <c r="E18" s="36" t="inlineStr">
+        <is>
+          <t>[MB-A R5] Shuttle Smashers vs The Feather Sailors</t>
+        </is>
+      </c>
+      <c r="F18" s="36" t="inlineStr">
+        <is>
+          <t>[W-B R5] Power Pair vs Double Trouble</t>
+        </is>
+      </c>
+      <c r="G18" s="36" t="inlineStr">
+        <is>
+          <t>[MB-B R5] Team Masala Dosa vs Shuttle Pirates</t>
+        </is>
+      </c>
+      <c r="H18" s="36" t="inlineStr">
+        <is>
+          <t>[W-B R5] Polka Dots vs Netique</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>13:40 - 14:00</t>
+        </is>
+      </c>
+      <c r="C19" s="34" t="inlineStr">
+        <is>
+          <t>[MB-B R5] Karnataka Knight Smashers vs R Squared</t>
+        </is>
+      </c>
+      <c r="D19" s="34" t="inlineStr">
+        <is>
           <t>[W-A R5] Phoenix Femmes vs Prime Strikers</t>
         </is>
       </c>
-      <c r="D18" s="36" t="inlineStr">
+      <c r="E19" s="34" t="inlineStr">
         <is>
           <t>[W-A R5] Cherry Champs vs Viva La Vida</t>
         </is>
       </c>
-      <c r="E18" s="36" t="inlineStr">
-        <is>
-          <t>[W-B R5] Power Pair vs Double Trouble</t>
-        </is>
-      </c>
-      <c r="F18" s="36" t="inlineStr">
-        <is>
-          <t>[W-B R5] Shuttlerz vs Netique</t>
-        </is>
-      </c>
-      <c r="G18" s="35" t="inlineStr"/>
-      <c r="H18" s="35" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="37" t="inlineStr">
-        <is>
-          <t>LUNCH BREAK (13:40 - 14:10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1" s="19"/>
-    <row r="21" ht="30" customHeight="1" s="19">
-      <c r="A21" s="26" t="inlineStr">
-        <is>
-          <t>Knockout Stage (14:10 - 16:45)</t>
-        </is>
-      </c>
-    </row>
+      <c r="F19" s="33" t="inlineStr"/>
+      <c r="G19" s="33" t="inlineStr"/>
+      <c r="H19" s="33" t="inlineStr"/>
+    </row>
+    <row r="20" ht="30" customHeight="1" s="19">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>LUNCH BREAK (14:00 - 14:30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1" s="19"/>
     <row r="22" ht="30" customHeight="1" s="19">
-      <c r="A22" s="32" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Knockout Stage (14:30 - 17:05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1" s="19">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Round</t>
         </is>
       </c>
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C22" s="32" t="inlineStr">
+      <c r="C23" s="32" t="inlineStr">
         <is>
           <t>Court 1</t>
         </is>
       </c>
-      <c r="D22" s="32" t="inlineStr">
+      <c r="D23" s="32" t="inlineStr">
         <is>
           <t>Court 2</t>
         </is>
       </c>
-      <c r="E22" s="32" t="inlineStr">
+      <c r="E23" s="32" t="inlineStr">
         <is>
           <t>Court 3</t>
         </is>
       </c>
-      <c r="F22" s="32" t="inlineStr">
+      <c r="F23" s="32" t="inlineStr">
         <is>
           <t>Court 4</t>
         </is>
       </c>
-      <c r="G22" s="32" t="inlineStr">
+      <c r="G23" s="32" t="inlineStr">
         <is>
           <t>Court 5</t>
         </is>
       </c>
-      <c r="H22" s="32" t="inlineStr">
+      <c r="H23" s="32" t="inlineStr">
         <is>
           <t>Court 6</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1" s="19">
-      <c r="A23" s="33" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>KO R1</t>
         </is>
       </c>
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t>14:10 - 14:45</t>
-        </is>
-      </c>
-      <c r="C23" s="34" t="inlineStr">
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>14:30 - 15:05</t>
+        </is>
+      </c>
+      <c r="C24" s="34" t="inlineStr">
         <is>
           <t>[MB QF1] MB-A Winner vs MB-D Runner-up</t>
         </is>
       </c>
-      <c r="D23" s="34" t="inlineStr">
+      <c r="D24" s="34" t="inlineStr">
         <is>
           <t>[MB QF2] MB-B Winner vs MB-C Runner-up</t>
         </is>
       </c>
-      <c r="E23" s="34" t="inlineStr">
+      <c r="E24" s="34" t="inlineStr">
         <is>
           <t>[MB QF3] MB-C Winner vs MB-B Runner-up</t>
         </is>
       </c>
-      <c r="F23" s="34" t="inlineStr">
+      <c r="F24" s="34" t="inlineStr">
         <is>
           <t>[MB QF4] MB-D Winner vs MB-A Runner-up</t>
         </is>
       </c>
-      <c r="G23" s="34" t="inlineStr">
+      <c r="G24" s="34" t="inlineStr">
         <is>
           <t>[MI QF1] MI-A Winner vs MI-D Runner-up</t>
         </is>
       </c>
-      <c r="H23" s="34" t="inlineStr">
+      <c r="H24" s="34" t="inlineStr">
         <is>
           <t>[MI QF2] MI-B Winner vs MI-C Runner-up</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="35" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="35" t="inlineStr">
         <is>
           <t>KO R2</t>
         </is>
       </c>
-      <c r="B24" s="35" t="inlineStr">
-        <is>
-          <t>14:50 - 15:25</t>
-        </is>
-      </c>
-      <c r="C24" s="36" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
+        <is>
+          <t>15:10 - 15:45</t>
+        </is>
+      </c>
+      <c r="C25" s="36" t="inlineStr">
         <is>
           <t>[MI QF3] MI-C Winner vs MI-B Runner-up</t>
         </is>
       </c>
-      <c r="D24" s="36" t="inlineStr">
+      <c r="D25" s="36" t="inlineStr">
         <is>
           <t>[MI QF4] MI-D Winner vs MI-A Runner-up</t>
         </is>
       </c>
-      <c r="E24" s="36" t="inlineStr">
+      <c r="E25" s="36" t="inlineStr">
         <is>
           <t>[W SF1] W-A Winner vs W-B Runner-up</t>
         </is>
       </c>
-      <c r="F24" s="36" t="inlineStr">
+      <c r="F25" s="36" t="inlineStr">
         <is>
           <t>[W SF2] W-B Winner vs W-A Runner-up</t>
         </is>
       </c>
-      <c r="G24" s="36" t="inlineStr">
+      <c r="G25" s="36" t="inlineStr">
         <is>
           <t>[MB SF1] MB QF1 Winner vs MB QF4 Winner</t>
         </is>
       </c>
-      <c r="H24" s="36" t="inlineStr">
+      <c r="H25" s="36" t="inlineStr">
         <is>
           <t>[MB SF2] MB QF2 Winner vs MB QF3 Winner</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="33" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t>KO R3</t>
         </is>
       </c>
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t>15:30 - 16:05</t>
-        </is>
-      </c>
-      <c r="C25" s="34" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>15:50 - 16:25</t>
+        </is>
+      </c>
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>[MI SF1] MI QF1 Winner vs MI QF4 Winner</t>
         </is>
       </c>
-      <c r="D25" s="34" t="inlineStr">
+      <c r="D26" s="34" t="inlineStr">
         <is>
           <t>[MI SF2] MI QF2 Winner vs MI QF3 Winner</t>
         </is>
       </c>
-      <c r="E25" s="34" t="inlineStr">
+      <c r="E26" s="34" t="inlineStr">
         <is>
           <t>[W FINAL] Women's Final: SF1 Winner vs SF2 Winner</t>
         </is>
       </c>
-      <c r="F25" s="34" t="inlineStr">
+      <c r="F26" s="34" t="inlineStr">
         <is>
           <t>[MB FINAL] Men's Beginner Final: SF1 Winner vs SF2 Winner</t>
         </is>
       </c>
-      <c r="G25" s="33" t="inlineStr"/>
-      <c r="H25" s="33" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="35" t="inlineStr">
+      <c r="G26" s="33" t="inlineStr"/>
+      <c r="H26" s="33" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="35" t="inlineStr">
         <is>
           <t>KO R4</t>
         </is>
       </c>
-      <c r="B26" s="35" t="inlineStr">
-        <is>
-          <t>16:10 - 16:45</t>
-        </is>
-      </c>
-      <c r="C26" s="36" t="inlineStr">
+      <c r="B27" s="35" t="inlineStr">
+        <is>
+          <t>16:30 - 17:05</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
         <is>
           <t>[MI FINAL] Men's Intermediate Final: SF1 Winner vs SF2 Winner</t>
         </is>
       </c>
-      <c r="D26" s="35" t="inlineStr"/>
-      <c r="E26" s="35" t="inlineStr"/>
-      <c r="F26" s="35" t="inlineStr"/>
-      <c r="G26" s="35" t="inlineStr"/>
-      <c r="H26" s="35" t="inlineStr"/>
+      <c r="D27" s="35" t="inlineStr"/>
+      <c r="E27" s="35" t="inlineStr"/>
+      <c r="F27" s="35" t="inlineStr"/>
+      <c r="G27" s="35" t="inlineStr"/>
+      <c r="H27" s="35" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6468,7 +6712,7 @@
       </c>
       <c r="D14" s="33" t="inlineStr">
         <is>
-          <t>Court 1</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr"/>
@@ -6492,7 +6736,7 @@
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr"/>
@@ -6516,7 +6760,7 @@
       </c>
       <c r="D16" s="33" t="inlineStr">
         <is>
-          <t>Court 1</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E16" s="33" t="inlineStr"/>
@@ -6535,12 +6779,12 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>11:20 - 11:40</t>
+          <t>11:40 - 12:00</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr"/>
@@ -6559,7 +6803,7 @@
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>12:20 - 12:40</t>
+          <t>12:40 - 13:00</t>
         </is>
       </c>
       <c r="D18" s="33" t="inlineStr">
@@ -6583,7 +6827,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>12:20 - 12:40</t>
+          <t>12:40 - 13:00</t>
         </is>
       </c>
       <c r="D19" s="33" t="inlineStr">
@@ -6607,7 +6851,7 @@
       </c>
       <c r="C20" s="33" t="inlineStr">
         <is>
-          <t>13:00 - 13:20</t>
+          <t>13:20 - 13:40</t>
         </is>
       </c>
       <c r="D20" s="33" t="inlineStr">
@@ -6631,12 +6875,12 @@
       </c>
       <c r="C21" s="33" t="inlineStr">
         <is>
-          <t>13:00 - 13:20</t>
+          <t>13:20 - 13:40</t>
         </is>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E21" s="33" t="inlineStr"/>
@@ -6840,12 +7084,12 @@
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
-          <t>09:20 - 09:40</t>
+          <t>09:40 - 10:00</t>
         </is>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 1</t>
         </is>
       </c>
       <c r="E34" s="33" t="inlineStr"/>
@@ -6864,12 +7108,12 @@
       </c>
       <c r="C35" s="33" t="inlineStr">
         <is>
-          <t>10:20 - 10:40</t>
+          <t>10:40 - 11:00</t>
         </is>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 1</t>
         </is>
       </c>
       <c r="E35" s="33" t="inlineStr"/>
@@ -6888,12 +7132,12 @@
       </c>
       <c r="C36" s="33" t="inlineStr">
         <is>
-          <t>10:20 - 10:40</t>
+          <t>10:40 - 11:00</t>
         </is>
       </c>
       <c r="D36" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E36" s="33" t="inlineStr"/>
@@ -6912,12 +7156,12 @@
       </c>
       <c r="C37" s="33" t="inlineStr">
         <is>
-          <t>11:20 - 11:40</t>
+          <t>11:40 - 12:00</t>
         </is>
       </c>
       <c r="D37" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 1</t>
         </is>
       </c>
       <c r="E37" s="33" t="inlineStr"/>
@@ -6936,12 +7180,12 @@
       </c>
       <c r="C38" s="33" t="inlineStr">
         <is>
-          <t>11:20 - 11:40</t>
+          <t>11:40 - 12:00</t>
         </is>
       </c>
       <c r="D38" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E38" s="33" t="inlineStr"/>
@@ -6960,7 +7204,7 @@
       </c>
       <c r="C39" s="33" t="inlineStr">
         <is>
-          <t>12:20 - 12:40</t>
+          <t>12:40 - 13:00</t>
         </is>
       </c>
       <c r="D39" s="33" t="inlineStr">
@@ -6984,7 +7228,7 @@
       </c>
       <c r="C40" s="33" t="inlineStr">
         <is>
-          <t>12:20 - 12:40</t>
+          <t>12:40 - 13:00</t>
         </is>
       </c>
       <c r="D40" s="33" t="inlineStr">
@@ -7008,12 +7252,12 @@
       </c>
       <c r="C41" s="33" t="inlineStr">
         <is>
-          <t>13:00 - 13:20</t>
+          <t>13:20 - 13:40</t>
         </is>
       </c>
       <c r="D41" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E41" s="33" t="inlineStr"/>
@@ -7032,12 +7276,12 @@
       </c>
       <c r="C42" s="33" t="inlineStr">
         <is>
-          <t>13:00 - 13:20</t>
+          <t>13:40 - 14:00</t>
         </is>
       </c>
       <c r="D42" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 1</t>
         </is>
       </c>
       <c r="E42" s="33" t="inlineStr"/>
@@ -7336,7 +7580,7 @@
       </c>
       <c r="D59" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E59" s="33" t="inlineStr"/>
@@ -7360,7 +7604,7 @@
       </c>
       <c r="D60" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E60" s="33" t="inlineStr"/>
@@ -7408,7 +7652,7 @@
       </c>
       <c r="D62" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E62" s="33" t="inlineStr"/>
@@ -7432,7 +7676,7 @@
       </c>
       <c r="D63" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E63" s="33" t="inlineStr"/>
@@ -7480,7 +7724,7 @@
       </c>
       <c r="D65" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E65" s="33" t="inlineStr"/>
@@ -7504,7 +7748,7 @@
       </c>
       <c r="D66" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E66" s="33" t="inlineStr"/>
@@ -7523,7 +7767,7 @@
       </c>
       <c r="C67" s="33" t="inlineStr">
         <is>
-          <t>12:40 - 13:00</t>
+          <t>13:00 - 13:20</t>
         </is>
       </c>
       <c r="D67" s="33" t="inlineStr">
@@ -7547,12 +7791,12 @@
       </c>
       <c r="C68" s="33" t="inlineStr">
         <is>
-          <t>12:40 - 13:00</t>
+          <t>13:00 - 13:20</t>
         </is>
       </c>
       <c r="D68" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E68" s="33" t="inlineStr"/>
@@ -7571,12 +7815,12 @@
       </c>
       <c r="C69" s="33" t="inlineStr">
         <is>
-          <t>12:40 - 13:00</t>
+          <t>13:00 - 13:20</t>
         </is>
       </c>
       <c r="D69" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E69" s="33" t="inlineStr"/>
@@ -7851,7 +8095,7 @@
       </c>
       <c r="D85" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E85" s="33" t="inlineStr"/>
@@ -7875,7 +8119,7 @@
       </c>
       <c r="D86" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E86" s="33" t="inlineStr"/>
@@ -7894,12 +8138,12 @@
       </c>
       <c r="C87" s="33" t="inlineStr">
         <is>
-          <t>10:00 - 10:20</t>
+          <t>10:20 - 10:40</t>
         </is>
       </c>
       <c r="D87" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 1</t>
         </is>
       </c>
       <c r="E87" s="33" t="inlineStr"/>
@@ -7923,7 +8167,7 @@
       </c>
       <c r="D88" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E88" s="33" t="inlineStr"/>
@@ -7942,12 +8186,12 @@
       </c>
       <c r="C89" s="33" t="inlineStr">
         <is>
-          <t>11:00 - 11:20</t>
+          <t>11:20 - 11:40</t>
         </is>
       </c>
       <c r="D89" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 1</t>
         </is>
       </c>
       <c r="E89" s="33" t="inlineStr"/>
@@ -7966,12 +8210,12 @@
       </c>
       <c r="C90" s="33" t="inlineStr">
         <is>
-          <t>11:00 - 11:20</t>
+          <t>11:20 - 11:40</t>
         </is>
       </c>
       <c r="D90" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E90" s="33" t="inlineStr"/>
@@ -7990,12 +8234,12 @@
       </c>
       <c r="C91" s="33" t="inlineStr">
         <is>
-          <t>12:00 - 12:20</t>
+          <t>12:20 - 12:40</t>
         </is>
       </c>
       <c r="D91" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 1</t>
         </is>
       </c>
       <c r="E91" s="33" t="inlineStr"/>
@@ -8014,12 +8258,12 @@
       </c>
       <c r="C92" s="33" t="inlineStr">
         <is>
-          <t>12:00 - 12:20</t>
+          <t>12:20 - 12:40</t>
         </is>
       </c>
       <c r="D92" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E92" s="33" t="inlineStr"/>
@@ -8038,12 +8282,12 @@
       </c>
       <c r="C93" s="33" t="inlineStr">
         <is>
-          <t>12:00 - 12:20</t>
+          <t>12:20 - 12:40</t>
         </is>
       </c>
       <c r="D93" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E93" s="33" t="inlineStr"/>
@@ -8062,12 +8306,12 @@
       </c>
       <c r="C94" s="33" t="inlineStr">
         <is>
-          <t>12:40 - 13:00</t>
+          <t>13:00 - 13:20</t>
         </is>
       </c>
       <c r="D94" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E94" s="33" t="inlineStr"/>
@@ -8124,9 +8368,9 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A72:F72"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8300,7 +8544,7 @@
       </c>
       <c r="D10" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E10" s="33" t="inlineStr"/>
@@ -8324,7 +8568,7 @@
       </c>
       <c r="D11" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E11" s="33" t="inlineStr"/>
@@ -8348,7 +8592,7 @@
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E12" s="33" t="inlineStr"/>
@@ -8497,7 +8741,7 @@
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E22" s="33" t="inlineStr"/>
@@ -8521,7 +8765,7 @@
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E23" s="33" t="inlineStr"/>
@@ -8540,12 +8784,12 @@
       </c>
       <c r="C24" s="33" t="inlineStr">
         <is>
-          <t>11:40 - 12:00</t>
+          <t>12:00 - 12:20</t>
         </is>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E24" s="33" t="inlineStr"/>
@@ -8694,7 +8938,7 @@
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E34" s="33" t="inlineStr"/>
@@ -8713,12 +8957,12 @@
       </c>
       <c r="C35" s="33" t="inlineStr">
         <is>
-          <t>10:40 - 11:00</t>
+          <t>11:00 - 11:20</t>
         </is>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E35" s="33" t="inlineStr"/>
@@ -8737,12 +8981,12 @@
       </c>
       <c r="C36" s="33" t="inlineStr">
         <is>
-          <t>11:40 - 12:00</t>
+          <t>12:00 - 12:20</t>
         </is>
       </c>
       <c r="D36" s="33" t="inlineStr">
         <is>
-          <t>Court 5</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E36" s="33" t="inlineStr"/>
@@ -8886,12 +9130,12 @@
       </c>
       <c r="C46" s="33" t="inlineStr">
         <is>
-          <t>09:40 - 10:00</t>
+          <t>10:00 - 10:20</t>
         </is>
       </c>
       <c r="D46" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E46" s="33" t="inlineStr"/>
@@ -8910,12 +9154,12 @@
       </c>
       <c r="C47" s="33" t="inlineStr">
         <is>
-          <t>10:40 - 11:00</t>
+          <t>11:00 - 11:20</t>
         </is>
       </c>
       <c r="D47" s="33" t="inlineStr">
         <is>
-          <t>Court 6</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E47" s="33" t="inlineStr"/>
@@ -8934,7 +9178,7 @@
       </c>
       <c r="C48" s="33" t="inlineStr">
         <is>
-          <t>11:40 - 12:00</t>
+          <t>12:00 - 12:20</t>
         </is>
       </c>
       <c r="D48" s="33" t="inlineStr">
@@ -8963,7 +9207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" style="19" min="1" max="1"/>
@@ -9155,7 +9399,7 @@
       </c>
       <c r="C12" s="33" t="inlineStr">
         <is>
-          <t>09:20 - 09:40</t>
+          <t>09:40 - 10:00</t>
         </is>
       </c>
       <c r="D12" s="33" t="inlineStr">
@@ -9179,7 +9423,7 @@
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>09:20 - 09:40</t>
+          <t>09:40 - 10:00</t>
         </is>
       </c>
       <c r="D13" s="33" t="inlineStr">
@@ -9203,7 +9447,7 @@
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>10:20 - 10:40</t>
+          <t>10:40 - 11:00</t>
         </is>
       </c>
       <c r="D14" s="33" t="inlineStr">
@@ -9227,12 +9471,12 @@
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
-          <t>10:20 - 10:40</t>
+          <t>10:40 - 11:00</t>
         </is>
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr"/>
@@ -9251,7 +9495,7 @@
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
-          <t>11:20 - 11:40</t>
+          <t>11:40 - 12:00</t>
         </is>
       </c>
       <c r="D16" s="33" t="inlineStr">
@@ -9275,12 +9519,12 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>11:20 - 11:40</t>
+          <t>11:40 - 12:00</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 5</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr"/>
@@ -9299,7 +9543,7 @@
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>12:20 - 12:40</t>
+          <t>12:40 - 13:00</t>
         </is>
       </c>
       <c r="D18" s="33" t="inlineStr">
@@ -9323,7 +9567,7 @@
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>12:20 - 12:40</t>
+          <t>12:40 - 13:00</t>
         </is>
       </c>
       <c r="D19" s="33" t="inlineStr">
@@ -9347,12 +9591,12 @@
       </c>
       <c r="C20" s="33" t="inlineStr">
         <is>
-          <t>13:20 - 13:40</t>
+          <t>13:40 - 14:00</t>
         </is>
       </c>
       <c r="D20" s="33" t="inlineStr">
         <is>
-          <t>Court 1</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E20" s="33" t="inlineStr"/>
@@ -9371,12 +9615,12 @@
       </c>
       <c r="C21" s="33" t="inlineStr">
         <is>
-          <t>13:20 - 13:40</t>
+          <t>13:40 - 14:00</t>
         </is>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 3</t>
         </is>
       </c>
       <c r="E21" s="33" t="inlineStr"/>
@@ -9511,61 +9755,55 @@
       <c r="E30" s="33" t="inlineStr"/>
       <c r="F30" s="33" t="inlineStr"/>
     </row>
-    <row r="32">
-      <c r="A32" s="32" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>Polka Dots</t>
+        </is>
+      </c>
+      <c r="C31" s="36" t="inlineStr">
+        <is>
+          <t>Himanshi Singh &amp; Chrisma Serrao</t>
+        </is>
+      </c>
+      <c r="D31" s="35" t="inlineStr"/>
+      <c r="E31" s="35" t="inlineStr"/>
+      <c r="F31" s="35" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>Round</t>
         </is>
       </c>
-      <c r="B32" s="32" t="inlineStr">
+      <c r="B33" s="32" t="inlineStr">
         <is>
           <t>Match-up</t>
         </is>
       </c>
-      <c r="C32" s="32" t="inlineStr">
+      <c r="C33" s="32" t="inlineStr">
         <is>
           <t>Scheduled Time</t>
         </is>
       </c>
-      <c r="D32" s="32" t="inlineStr">
+      <c r="D33" s="32" t="inlineStr">
         <is>
           <t>Court</t>
         </is>
       </c>
-      <c r="E32" s="32" t="inlineStr">
+      <c r="E33" s="32" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="F32" s="32" t="inlineStr">
+      <c r="F33" s="32" t="inlineStr">
         <is>
           <t>Winner</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="33" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B33" s="34" t="inlineStr">
-        <is>
-          <t>Racquet Rebels  vs  Power Pair</t>
-        </is>
-      </c>
-      <c r="C33" s="33" t="inlineStr">
-        <is>
-          <t>09:40 - 10:00</t>
-        </is>
-      </c>
-      <c r="D33" s="33" t="inlineStr">
-        <is>
-          <t>Court 1</t>
-        </is>
-      </c>
-      <c r="E33" s="33" t="inlineStr"/>
-      <c r="F33" s="33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="33" t="inlineStr">
@@ -9575,17 +9813,17 @@
       </c>
       <c r="B34" s="34" t="inlineStr">
         <is>
-          <t>Shuttlerz  vs  Double Trouble</t>
+          <t>Racquet Rebels  vs  Power Pair</t>
         </is>
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
-          <t>09:40 - 10:00</t>
+          <t>09:20 - 09:40</t>
         </is>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E34" s="33" t="inlineStr"/>
@@ -9594,22 +9832,22 @@
     <row r="35">
       <c r="A35" s="33" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B35" s="34" t="inlineStr">
         <is>
-          <t>Racquet Rebels  vs  Shuttlerz</t>
+          <t>Polka Dots  vs  Shuttlerz</t>
         </is>
       </c>
       <c r="C35" s="33" t="inlineStr">
         <is>
-          <t>10:40 - 11:00</t>
+          <t>09:20 - 09:40</t>
         </is>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
-          <t>Court 1</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E35" s="33" t="inlineStr"/>
@@ -9618,22 +9856,22 @@
     <row r="36">
       <c r="A36" s="33" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B36" s="34" t="inlineStr">
         <is>
-          <t>Double Trouble  vs  Netique</t>
+          <t>Netique  vs  Double Trouble</t>
         </is>
       </c>
       <c r="C36" s="33" t="inlineStr">
         <is>
-          <t>10:40 - 11:00</t>
+          <t>09:20 - 09:40</t>
         </is>
       </c>
       <c r="D36" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E36" s="33" t="inlineStr"/>
@@ -9642,22 +9880,22 @@
     <row r="37">
       <c r="A37" s="33" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>Racquet Rebels  vs  Double Trouble</t>
+          <t>Racquet Rebels  vs  Polka Dots</t>
         </is>
       </c>
       <c r="C37" s="33" t="inlineStr">
         <is>
-          <t>11:40 - 12:00</t>
+          <t>10:20 - 10:40</t>
         </is>
       </c>
       <c r="D37" s="33" t="inlineStr">
         <is>
-          <t>Court 1</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E37" s="33" t="inlineStr"/>
@@ -9666,22 +9904,22 @@
     <row r="38">
       <c r="A38" s="33" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B38" s="34" t="inlineStr">
         <is>
-          <t>Power Pair  vs  Netique</t>
+          <t>Netique  vs  Power Pair</t>
         </is>
       </c>
       <c r="C38" s="33" t="inlineStr">
         <is>
-          <t>11:40 - 12:00</t>
+          <t>10:20 - 10:40</t>
         </is>
       </c>
       <c r="D38" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E38" s="33" t="inlineStr"/>
@@ -9690,22 +9928,22 @@
     <row r="39">
       <c r="A39" s="33" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B39" s="34" t="inlineStr">
         <is>
-          <t>Racquet Rebels  vs  Netique</t>
+          <t>Double Trouble  vs  Shuttlerz</t>
         </is>
       </c>
       <c r="C39" s="33" t="inlineStr">
         <is>
-          <t>12:40 - 13:00</t>
+          <t>10:20 - 10:40</t>
         </is>
       </c>
       <c r="D39" s="33" t="inlineStr">
         <is>
-          <t>Court 2</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E39" s="33" t="inlineStr"/>
@@ -9714,22 +9952,22 @@
     <row r="40">
       <c r="A40" s="33" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B40" s="34" t="inlineStr">
         <is>
-          <t>Power Pair  vs  Shuttlerz</t>
+          <t>Racquet Rebels  vs  Netique</t>
         </is>
       </c>
       <c r="C40" s="33" t="inlineStr">
         <is>
-          <t>12:40 - 13:00</t>
+          <t>11:20 - 11:40</t>
         </is>
       </c>
       <c r="D40" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 2</t>
         </is>
       </c>
       <c r="E40" s="33" t="inlineStr"/>
@@ -9738,22 +9976,22 @@
     <row r="41">
       <c r="A41" s="33" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>Power Pair  vs  Double Trouble</t>
+          <t>Double Trouble  vs  Polka Dots</t>
         </is>
       </c>
       <c r="C41" s="33" t="inlineStr">
         <is>
-          <t>13:20 - 13:40</t>
+          <t>11:20 - 11:40</t>
         </is>
       </c>
       <c r="D41" s="33" t="inlineStr">
         <is>
-          <t>Court 3</t>
+          <t>Court 4</t>
         </is>
       </c>
       <c r="E41" s="33" t="inlineStr"/>
@@ -9762,26 +10000,170 @@
     <row r="42">
       <c r="A42" s="33" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B42" s="34" t="inlineStr">
         <is>
-          <t>Shuttlerz  vs  Netique</t>
+          <t>Shuttlerz  vs  Power Pair</t>
         </is>
       </c>
       <c r="C42" s="33" t="inlineStr">
         <is>
-          <t>13:20 - 13:40</t>
+          <t>11:20 - 11:40</t>
         </is>
       </c>
       <c r="D42" s="33" t="inlineStr">
         <is>
-          <t>Court 4</t>
+          <t>Court 6</t>
         </is>
       </c>
       <c r="E42" s="33" t="inlineStr"/>
       <c r="F42" s="33" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="33" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B43" s="34" t="inlineStr">
+        <is>
+          <t>Racquet Rebels  vs  Double Trouble</t>
+        </is>
+      </c>
+      <c r="C43" s="33" t="inlineStr">
+        <is>
+          <t>12:20 - 12:40</t>
+        </is>
+      </c>
+      <c r="D43" s="33" t="inlineStr">
+        <is>
+          <t>Court 2</t>
+        </is>
+      </c>
+      <c r="E43" s="33" t="inlineStr"/>
+      <c r="F43" s="33" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="33" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B44" s="34" t="inlineStr">
+        <is>
+          <t>Shuttlerz  vs  Netique</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>12:20 - 12:40</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>Court 4</t>
+        </is>
+      </c>
+      <c r="E44" s="33" t="inlineStr"/>
+      <c r="F44" s="33" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="33" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B45" s="34" t="inlineStr">
+        <is>
+          <t>Polka Dots  vs  Power Pair</t>
+        </is>
+      </c>
+      <c r="C45" s="33" t="inlineStr">
+        <is>
+          <t>12:20 - 12:40</t>
+        </is>
+      </c>
+      <c r="D45" s="33" t="inlineStr">
+        <is>
+          <t>Court 6</t>
+        </is>
+      </c>
+      <c r="E45" s="33" t="inlineStr"/>
+      <c r="F45" s="33" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="33" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B46" s="34" t="inlineStr">
+        <is>
+          <t>Racquet Rebels  vs  Shuttlerz</t>
+        </is>
+      </c>
+      <c r="C46" s="33" t="inlineStr">
+        <is>
+          <t>13:20 - 13:40</t>
+        </is>
+      </c>
+      <c r="D46" s="33" t="inlineStr">
+        <is>
+          <t>Court 2</t>
+        </is>
+      </c>
+      <c r="E46" s="33" t="inlineStr"/>
+      <c r="F46" s="33" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="33" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B47" s="34" t="inlineStr">
+        <is>
+          <t>Power Pair  vs  Double Trouble</t>
+        </is>
+      </c>
+      <c r="C47" s="33" t="inlineStr">
+        <is>
+          <t>13:20 - 13:40</t>
+        </is>
+      </c>
+      <c r="D47" s="33" t="inlineStr">
+        <is>
+          <t>Court 4</t>
+        </is>
+      </c>
+      <c r="E47" s="33" t="inlineStr"/>
+      <c r="F47" s="33" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="33" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B48" s="34" t="inlineStr">
+        <is>
+          <t>Polka Dots  vs  Netique</t>
+        </is>
+      </c>
+      <c r="C48" s="33" t="inlineStr">
+        <is>
+          <t>13:20 - 13:40</t>
+        </is>
+      </c>
+      <c r="D48" s="33" t="inlineStr">
+        <is>
+          <t>Court 6</t>
+        </is>
+      </c>
+      <c r="E48" s="33" t="inlineStr"/>
+      <c r="F48" s="33" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -9864,7 +10246,7 @@
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>14:10 - 14:45</t>
+          <t>14:30 - 15:05</t>
         </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
@@ -9888,7 +10270,7 @@
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>14:10 - 14:45</t>
+          <t>14:30 - 15:05</t>
         </is>
       </c>
       <c r="C6" s="35" t="inlineStr">
@@ -9912,7 +10294,7 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>14:10 - 14:45</t>
+          <t>14:30 - 15:05</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
@@ -9936,7 +10318,7 @@
       </c>
       <c r="B8" s="35" t="inlineStr">
         <is>
-          <t>14:10 - 14:45</t>
+          <t>14:30 - 15:05</t>
         </is>
       </c>
       <c r="C8" s="35" t="inlineStr">
@@ -9960,7 +10342,7 @@
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>14:50 - 15:25</t>
+          <t>15:10 - 15:45</t>
         </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
@@ -9984,7 +10366,7 @@
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>14:50 - 15:25</t>
+          <t>15:10 - 15:45</t>
         </is>
       </c>
       <c r="C10" s="35" t="inlineStr">
@@ -10008,7 +10390,7 @@
       </c>
       <c r="B11" s="38" t="inlineStr">
         <is>
-          <t>15:30 - 16:05</t>
+          <t>15:50 - 16:25</t>
         </is>
       </c>
       <c r="C11" s="38" t="inlineStr">
@@ -10071,7 +10453,7 @@
       </c>
       <c r="B16" s="33" t="inlineStr">
         <is>
-          <t>14:10 - 14:45</t>
+          <t>14:30 - 15:05</t>
         </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
@@ -10095,7 +10477,7 @@
       </c>
       <c r="B17" s="35" t="inlineStr">
         <is>
-          <t>14:10 - 14:45</t>
+          <t>14:30 - 15:05</t>
         </is>
       </c>
       <c r="C17" s="35" t="inlineStr">
@@ -10119,7 +10501,7 @@
       </c>
       <c r="B18" s="33" t="inlineStr">
         <is>
-          <t>14:50 - 15:25</t>
+          <t>15:10 - 15:45</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
@@ -10143,7 +10525,7 @@
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>14:50 - 15:25</t>
+          <t>15:10 - 15:45</t>
         </is>
       </c>
       <c r="C19" s="35" t="inlineStr">
@@ -10167,7 +10549,7 @@
       </c>
       <c r="B20" s="33" t="inlineStr">
         <is>
-          <t>15:30 - 16:05</t>
+          <t>15:50 - 16:25</t>
         </is>
       </c>
       <c r="C20" s="33" t="inlineStr">
@@ -10191,7 +10573,7 @@
       </c>
       <c r="B21" s="35" t="inlineStr">
         <is>
-          <t>15:30 - 16:05</t>
+          <t>15:50 - 16:25</t>
         </is>
       </c>
       <c r="C21" s="35" t="inlineStr">
@@ -10215,7 +10597,7 @@
       </c>
       <c r="B22" s="38" t="inlineStr">
         <is>
-          <t>16:10 - 16:45</t>
+          <t>16:30 - 17:05</t>
         </is>
       </c>
       <c r="C22" s="38" t="inlineStr">
@@ -10278,7 +10660,7 @@
       </c>
       <c r="B27" s="33" t="inlineStr">
         <is>
-          <t>14:50 - 15:25</t>
+          <t>15:10 - 15:45</t>
         </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
@@ -10302,7 +10684,7 @@
       </c>
       <c r="B28" s="35" t="inlineStr">
         <is>
-          <t>14:50 - 15:25</t>
+          <t>15:10 - 15:45</t>
         </is>
       </c>
       <c r="C28" s="35" t="inlineStr">
@@ -10326,7 +10708,7 @@
       </c>
       <c r="B29" s="38" t="inlineStr">
         <is>
-          <t>15:30 - 16:05</t>
+          <t>15:50 - 16:25</t>
         </is>
       </c>
       <c r="C29" s="38" t="inlineStr">

</xml_diff>